<commit_message>
Make plant Linkage type editable via dropdown
Replaces the read-only Linkage/Bridge Linkage tag with a <select>,
persisted through the existing overrides localStorage mechanism (same
one used for Current VC/Rakes) - no new persistence system, no backend
changes, linkage is never sent in the /optimize payload.

- buildState(): resolves a plant-level override (key
  "<plant>||__plant__") the same way per-source overrides already work
- renderPanel(): tag -> <select>, plus one change listener that updates
  state, calls the existing saveOverride(), and re-renders

Reset to source data clears it for free, since it shares clearOverrides().
</commit_message>
<xml_diff>
--- a/output/output.xlsx
+++ b/output/output.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Greedy (PREVIEW - not official)</t>
+          <t>OR-Tools</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">

</xml_diff>

<commit_message>
Add optional RSD/VC threshold support across schema, optimizer, and dashboard
</commit_message>
<xml_diff>
--- a/output/output.xlsx
+++ b/output/output.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,62 +417,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Plant</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Original Rakes</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Daily Available Rakes</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Optimized Rakes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Frozen</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Result Type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Old VC (plant)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>New VC (plant)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target VC</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Target Status (preview)</t>
         </is>

</xml_diff>

<commit_message>
Polish dashboard UI: UPRVUNL branding lockup, consistent card spacing, responsive layout
</commit_message>
<xml_diff>
--- a/output/output.xlsx
+++ b/output/output.xlsx
@@ -589,10 +589,10 @@
         <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F4" t="b">
         <v>0</v>
@@ -611,7 +611,7 @@
         <v>4.02</v>
       </c>
       <c r="J4" t="n">
-        <v>3.685</v>
+        <v>3.6775</v>
       </c>
       <c r="K4" t="n">
         <v>3.99</v>
@@ -659,7 +659,7 @@
         <v>4.02</v>
       </c>
       <c r="J5" t="n">
-        <v>3.685</v>
+        <v>3.6775</v>
       </c>
       <c r="K5" t="n">
         <v>3.99</v>
@@ -688,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
@@ -707,7 +707,7 @@
         <v>4.02</v>
       </c>
       <c r="J6" t="n">
-        <v>3.685</v>
+        <v>3.6775</v>
       </c>
       <c r="K6" t="n">
         <v>3.99</v>
@@ -755,7 +755,7 @@
         <v>4.02</v>
       </c>
       <c r="J7" t="n">
-        <v>3.685</v>
+        <v>3.6775</v>
       </c>
       <c r="K7" t="n">
         <v>3.99</v>
@@ -781,10 +781,10 @@
         <v>60</v>
       </c>
       <c r="D8" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E8" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -803,7 +803,7 @@
         <v>3.83</v>
       </c>
       <c r="J8" t="n">
-        <v>3.7807</v>
+        <v>3.81</v>
       </c>
       <c r="K8" t="n">
         <v>3.99</v>
@@ -829,10 +829,10 @@
         <v>25</v>
       </c>
       <c r="D9" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" t="n">
         <v>30</v>
-      </c>
-      <c r="E9" t="n">
-        <v>36</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
@@ -851,7 +851,7 @@
         <v>3.83</v>
       </c>
       <c r="J9" t="n">
-        <v>3.7807</v>
+        <v>3.81</v>
       </c>
       <c r="K9" t="n">
         <v>3.99</v>
@@ -899,7 +899,7 @@
         <v>3.83</v>
       </c>
       <c r="J10" t="n">
-        <v>3.7807</v>
+        <v>3.81</v>
       </c>
       <c r="K10" t="n">
         <v>3.99</v>

</xml_diff>